<commit_message>
refactor/clean codes and structures & add processing times
</commit_message>
<xml_diff>
--- a/outputs/results/phase11_hybrid_predictions.xlsx
+++ b/outputs/results/phase11_hybrid_predictions.xlsx
@@ -448,10 +448,10 @@
         <v>0.413</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5683102186266122</v>
+        <v>0.5229269835600924</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1553102186266123</v>
+        <v>0.1099269835600924</v>
       </c>
     </row>
     <row r="3">
@@ -464,10 +464,10 @@
         <v>0.413</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5611536524467602</v>
+        <v>0.4996169597505685</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1481536524467602</v>
+        <v>0.08661695975056849</v>
       </c>
     </row>
     <row r="4">
@@ -480,10 +480,10 @@
         <v>0.413</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5653618398902672</v>
+        <v>0.5975609020305078</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1523618398902672</v>
+        <v>0.1845609020305078</v>
       </c>
     </row>
     <row r="5">
@@ -496,10 +496,10 @@
         <v>0.413</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5054391157731151</v>
+        <v>0.5083672534013597</v>
       </c>
       <c r="D5" t="n">
-        <v>0.09243911577311509</v>
+        <v>0.09536725340135971</v>
       </c>
     </row>
     <row r="6">
@@ -512,10 +512,10 @@
         <v>0.5610000000000001</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6988138851465996</v>
+        <v>0.6559302857142858</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1378138851465995</v>
+        <v>0.09493028571428574</v>
       </c>
     </row>
     <row r="7">
@@ -528,10 +528,10 @@
         <v>0.5610000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5443113866332079</v>
+        <v>0.5203449012059372</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01668861336679217</v>
+        <v>0.04065509879406282</v>
       </c>
     </row>
     <row r="8">
@@ -544,10 +544,10 @@
         <v>0.5610000000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>0.509360492610563</v>
+        <v>0.6548735179859816</v>
       </c>
       <c r="D8" t="n">
-        <v>0.05163950738943701</v>
+        <v>0.09387351798598154</v>
       </c>
     </row>
     <row r="9">
@@ -560,10 +560,10 @@
         <v>0.5610000000000001</v>
       </c>
       <c r="C9" t="n">
-        <v>0.4368728355890162</v>
+        <v>0.4977730775097923</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1241271644109838</v>
+        <v>0.06322692249020778</v>
       </c>
     </row>
     <row r="10">
@@ -576,10 +576,10 @@
         <v>0.821</v>
       </c>
       <c r="C10" t="n">
-        <v>0.7005398080332383</v>
+        <v>0.4734660527210903</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1204601919667616</v>
+        <v>0.3475339472789096</v>
       </c>
     </row>
     <row r="11">
@@ -592,10 +592,10 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="C11" t="n">
-        <v>0.6481080945602008</v>
+        <v>0.6968840620490631</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1688919054397992</v>
+        <v>0.1201159379509369</v>
       </c>
     </row>
     <row r="12">
@@ -608,10 +608,10 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>0.5325945224140947</v>
+        <v>0.856325107967429</v>
       </c>
       <c r="D12" t="n">
-        <v>0.2844054775859053</v>
+        <v>0.03932510796742905</v>
       </c>
     </row>
     <row r="13">
@@ -624,10 +624,10 @@
         <v>1.381</v>
       </c>
       <c r="C13" t="n">
-        <v>0.571068406676654</v>
+        <v>0.6633635455576168</v>
       </c>
       <c r="D13" t="n">
-        <v>0.809931593323346</v>
+        <v>0.7176364544423832</v>
       </c>
     </row>
     <row r="14">
@@ -640,10 +640,10 @@
         <v>0.141</v>
       </c>
       <c r="C14" t="n">
-        <v>0.719616346938778</v>
+        <v>0.6254099773242631</v>
       </c>
       <c r="D14" t="n">
-        <v>0.5786163469387779</v>
+        <v>0.4844099773242631</v>
       </c>
     </row>
     <row r="15">
@@ -656,10 +656,10 @@
         <v>0.388</v>
       </c>
       <c r="C15" t="n">
-        <v>0.4995894693203616</v>
+        <v>0.624816035611215</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1115894693203616</v>
+        <v>0.236816035611215</v>
       </c>
     </row>
     <row r="16">
@@ -672,10 +672,10 @@
         <v>0.384</v>
       </c>
       <c r="C16" t="n">
-        <v>0.7928289016657935</v>
+        <v>0.6100571651721272</v>
       </c>
       <c r="D16" t="n">
-        <v>0.4088289016657934</v>
+        <v>0.2260571651721272</v>
       </c>
     </row>
     <row r="17">
@@ -688,10 +688,10 @@
         <v>0.384</v>
       </c>
       <c r="C17" t="n">
-        <v>0.7209558044733038</v>
+        <v>0.6586504862914854</v>
       </c>
       <c r="D17" t="n">
-        <v>0.3369558044733038</v>
+        <v>0.2746504862914854</v>
       </c>
     </row>
     <row r="18">
@@ -704,10 +704,10 @@
         <v>0.651</v>
       </c>
       <c r="C18" t="n">
-        <v>0.753822916218701</v>
+        <v>0.9401040459183673</v>
       </c>
       <c r="D18" t="n">
-        <v>0.102822916218701</v>
+        <v>0.2891040459183672</v>
       </c>
     </row>
     <row r="19">
@@ -720,10 +720,10 @@
         <v>0.429</v>
       </c>
       <c r="C19" t="n">
-        <v>0.6922074022683649</v>
+        <v>0.5688907611832613</v>
       </c>
       <c r="D19" t="n">
-        <v>0.2632074022683649</v>
+        <v>0.1398907611832613</v>
       </c>
     </row>
     <row r="20">
@@ -736,10 +736,10 @@
         <v>1.791</v>
       </c>
       <c r="C20" t="n">
-        <v>1.505114204045958</v>
+        <v>1.438098704081637</v>
       </c>
       <c r="D20" t="n">
-        <v>0.2858857959540417</v>
+        <v>0.3529012959183633</v>
       </c>
     </row>
     <row r="21">
@@ -752,10 +752,10 @@
         <v>2.331</v>
       </c>
       <c r="C21" t="n">
-        <v>2.507403902855065</v>
+        <v>2.661255639455761</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1764039028550646</v>
+        <v>0.3302556394557614</v>
       </c>
     </row>
     <row r="22">
@@ -768,10 +768,10 @@
         <v>0.667</v>
       </c>
       <c r="C22" t="n">
-        <v>0.5490446030715314</v>
+        <v>0.7480014427952999</v>
       </c>
       <c r="D22" t="n">
-        <v>0.1179553969284687</v>
+        <v>0.08100144279529986</v>
       </c>
     </row>
     <row r="23">
@@ -784,10 +784,10 @@
         <v>6.001</v>
       </c>
       <c r="C23" t="n">
-        <v>1.686722602219208</v>
+        <v>1.77919428571428</v>
       </c>
       <c r="D23" t="n">
-        <v>4.314277397780792</v>
+        <v>4.22180571428572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>